<commit_message>
Aggiunte altre fonti in bibliografia. Aggiunta una pagina al foglio excel con gli esperimenti in ordine 'analogo-cronologico'. Aggiunti dei commenti al libro di Righi
</commit_message>
<xml_diff>
--- a/lista_esperienze_utili.xlsx
+++ b/lista_esperienze_utili.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\monon\Desktop\tesi_magistrale_augusto_righi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{933C8C49-0716-47E3-A010-F8FF40418A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66EF896D-406A-45B9-A719-4EABE074F0C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{66EA259D-F02F-4B4B-8D79-75807FB00DE3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{66EA259D-F02F-4B4B-8D79-75807FB00DE3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
+    <sheet name="Esperienze_ordine_numerico" sheetId="1" r:id="rId1"/>
+    <sheet name="esperienze_ordine_storico" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="44">
   <si>
     <t>interferenza</t>
   </si>
@@ -79,9 +80,6 @@
     <t>§21 Interferenza</t>
   </si>
   <si>
-    <t>§22 Specchi di Frsenel</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Fresnel (1816–1819, </t>
     </r>
@@ -163,7 +161,55 @@
     <t>riflessione</t>
   </si>
   <si>
-    <t>esperienza di Hertz</t>
+    <t>§22 Specchi di Fresnel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">esperienza di Hertz, V. Lang (Wied. Ann. 1896 , b. LVII , p . 430 .), Lodge, Quincke, </t>
+  </si>
+  <si>
+    <t>Capitolo VI</t>
+  </si>
+  <si>
+    <t>§ 45 Prisma, lastra a facce parallele, lenti</t>
+  </si>
+  <si>
+    <t>rifrazione</t>
+  </si>
+  <si>
+    <t>Hertz, Lodge e Howard</t>
+  </si>
+  <si>
+    <t>Capitolo VII</t>
+  </si>
+  <si>
+    <t>§ 50 Doppia rifrazione prodotta dal legno</t>
+  </si>
+  <si>
+    <t>birifrangenza</t>
+  </si>
+  <si>
+    <t>Righi (Mem. della R. Acc. di Bologna, serie V, t. IV, pag. 487.), Mack (Wied. Ann. 1895 , b. LIV, p. 342.), Garbasso (Atti della R. Acc. di Torino , v. XXX , 19 maggio 1895.), Lebedew (Wied. Ann. 1895 , b. LVI , p . 1 .), J. C. Bose (Naturw. Rundschau 1896 , р. 191.)</t>
+  </si>
+  <si>
+    <t>I°</t>
+  </si>
+  <si>
+    <t>Numero esperimento (ordine storico)</t>
+  </si>
+  <si>
+    <t>II°</t>
+  </si>
+  <si>
+    <t>III°</t>
+  </si>
+  <si>
+    <t>IV°</t>
+  </si>
+  <si>
+    <t>V°</t>
+  </si>
+  <si>
+    <t>VI°</t>
   </si>
 </sst>
 </file>
@@ -179,13 +225,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <u/>
       <sz val="16"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -210,6 +249,12 @@
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -265,22 +310,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -595,169 +645,489 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12F48E3E-5622-4291-B85C-ABBDFC55B237}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="87.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="163" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="87.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.77734375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="163" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2">
+        <v>92</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="2">
+        <v>96</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2">
+        <v>106</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="2">
+        <v>108</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="3">
-        <v>92</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="3">
-        <v>96</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="3">
-        <v>106</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="5" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A8" s="3" t="s">
+      <c r="B8" s="2">
+        <v>116</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="3">
-        <v>116</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="3" t="s">
+    </row>
+    <row r="9" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A9" s="5" t="s">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A10" s="3" t="s">
+      <c r="B10" s="2">
+        <v>122</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="3">
-        <v>122</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="3" t="s">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A11" s="3" t="s">
+      <c r="B11" s="2">
+        <v>123</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="3">
-        <v>123</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="3" t="s">
+    </row>
+    <row r="12" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A12" s="5" t="s">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+    </row>
+    <row r="14" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A14" s="5" t="s">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A15" s="3" t="s">
+      <c r="B15" s="2">
+        <v>148</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B15" s="3">
-        <v>148</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="2" t="s">
         <v>28</v>
       </c>
     </row>
+    <row r="16" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="2">
+        <v>170</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A19" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="2">
+        <v>185</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9854597-87EB-4C33-BBAB-426A1C3FF53F}">
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="87.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.77734375" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="255.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="6">
+        <v>148</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+    </row>
+    <row r="5" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="6">
+        <v>170</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+    </row>
+    <row r="7" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="6">
+        <v>122</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="6">
+        <v>123</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A9" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+    </row>
+    <row r="10" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="6">
+        <v>185</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A11" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+    </row>
+    <row r="12" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6">
+        <v>92</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" s="6">
+        <v>96</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="6">
+        <v>106</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="6">
+        <v>108</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A16" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+    </row>
+    <row r="17" spans="1:4" ht="21" x14ac:dyDescent="0.4">
+      <c r="A17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="6">
+        <v>116</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="21" x14ac:dyDescent="0.4">
+      <c r="A18" s="2"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A19" s="3"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" spans="1:4" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A20" s="3"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="3"/>
+    </row>
+    <row r="22" spans="1:4" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A22" s="3"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="3"/>
+    </row>
+    <row r="25" spans="1:4" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A25" s="3"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="3"/>
+    </row>
+    <row r="26" spans="1:4" ht="21" x14ac:dyDescent="0.4">
+      <c r="A26" s="2"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="2"/>
+    </row>
+    <row r="27" spans="1:4" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A27" s="3"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="3"/>
+    </row>
+    <row r="29" spans="1:4" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="A29" s="3"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="3"/>
+    </row>
+    <row r="31" spans="1:4" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
aggiunte delle immagini per l'esperienza 38 (riflessione).
</commit_message>
<xml_diff>
--- a/lista_esperienze_utili.xlsx
+++ b/lista_esperienze_utili.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\monon\Desktop\tesi_magistrale_augusto_righi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66EF896D-406A-45B9-A719-4EABE074F0C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B110C89A-2E87-408E-BECB-D6F54D7404C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{66EA259D-F02F-4B4B-8D79-75807FB00DE3}"/>
   </bookViews>
@@ -879,7 +879,7 @@
     <col min="4" max="4" width="255.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
@@ -900,7 +900,7 @@
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
     </row>
-    <row r="3" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>25</v>
       </c>
@@ -921,7 +921,7 @@
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
     </row>
-    <row r="5" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>30</v>
       </c>
@@ -942,7 +942,7 @@
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
     </row>
-    <row r="7" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -956,7 +956,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
@@ -977,7 +977,7 @@
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
     </row>
-    <row r="10" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>34</v>
       </c>
@@ -998,7 +998,7 @@
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
     </row>
-    <row r="12" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
@@ -1012,7 +1012,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
@@ -1026,7 +1026,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>8</v>
       </c>
@@ -1040,7 +1040,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:4" customFormat="1" ht="21" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>10</v>
       </c>

</xml_diff>